<commit_message>
Scrum: actualización y corrección de archivos
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/2. Metodología Scrum/SPRINTS/SITRAFO_Sprint2_Burndown.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/2. Metodología Scrum/SPRINTS/SITRAFO_Sprint2_Burndown.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admusuario\Documents\SITRAFO\Fase 2\Evidencias Proyecto\Evidencias de documentación\2. Metodología Scrum\SPRINTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCE6BCFE-58F0-4FF8-9B85-3D47114DF7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96ED9C72-9FB8-469E-B3AA-00BD4C5981F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1235,7 +1235,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="5">
-        <f t="shared" ref="M5:M14" si="0">SUM(C5:L5)</f>
+        <f t="shared" ref="M5:M10" si="0">SUM(C5:L5)</f>
         <v>12</v>
       </c>
       <c r="N5" s="5"/>

</xml_diff>